<commit_message>
Rename SQAG storage namespace
</commit_message>
<xml_diff>
--- a/templates/quote-layout/quotation-layout.xlsx
+++ b/templates/quote-layout/quotation-layout.xlsx
@@ -1340,8 +1340,8 @@
 </worksheet>
 </file>
 
-<file path=customXml/kqag-layout-rules.xml><?xml version="1.0" encoding="utf-8"?>
-<layoutRules xmlns="https://swooshz.com/kqag/layout-rules/v1" schema="swooshz.quote-layout-rules.v1">
+<file path=customXml/sqag-layout-rules.xml><?xml version="1.0" encoding="utf-8"?>
+<layoutRules xmlns="https://swooshz.com/sqag/layout-rules/v1" schema="swooshz.quote-layout-rules.v1">
   <json>{"company_details":{"align_details_to_logo_left":true,"blank_line_before_bank_detail":true,"details_alignment":"left","details_below_logo":true,"details_first_page_only":true,"details_font_size_pt":9,"keep_logo_and_details_inside_print_area":true,"print_area_columns":"A:I"},"header":{"client_block":{"alignment":"left","fields":["client.name","client.address","client.attention","client.title","quote_date","project.title"],"position":"top-left"},"company_block":{"alignment":"left","position":"top-right","repeat_logo_on_continuation_pages":true,"show_details_on_first_page_only":true}},"line_items":{"bold_headers":true,"columns":["Pos.","Quantity","Service","Estimate"],"detail_rows":{"allowed_display_prices":["numeric","FOC","Included"],"number_format":"0.0"},"estimate_alignment":"right","numeric_price_format":"#,##0.00","quantity_alignment":"center","quantity_column_must_fit_examples":["24 m length","36 sqm"],"section_rows":{"amount_mode":"itemized_by_default","number_format":"0.0"},"show_internal_costs":false,"square_metre_unit":"sqm"},"output":{"currency":"SGD","master_format":"xlsx","pdf_default":"disabled"},"profile_id":"default","schema_version":1,"security":{"escape_formula_prefixes":["'=","'+","'-","'@"],"frontend_exposes_internal_pricing":false,"treat_text_as_untrusted_spreadsheet_text":true},"template":{"print_area_columns":"A:I","workbook":"quotation-layout.xlsx","worksheet":"Quotation"},"terms_notes_signature":{"acceptance_block_separate_from_notes":true,"company_signatory_title_below_name":true,"customer_acceptance_text_separate_from_terms":true,"notes_numbering":"plain_sequential","payment_terms_bold":true,"signature_blocks":["company","customer"]},"totals":{"border_scope":["label","amount","currency"],"keep_rows_together":true,"labels":["Total","Quote-level tax label and rate","Total including selected tax label"],"use_strong_bottom_rule_under_final_total":true,"use_top_rule_above_final_total":true,"use_top_rule_above_total":true}}</json>
 </layoutRules>
 </file>
</xml_diff>

<commit_message>
Rename SQAG storage namespace (#122)
</commit_message>
<xml_diff>
--- a/templates/quote-layout/quotation-layout.xlsx
+++ b/templates/quote-layout/quotation-layout.xlsx
@@ -1340,8 +1340,8 @@
 </worksheet>
 </file>
 
-<file path=customXml/kqag-layout-rules.xml><?xml version="1.0" encoding="utf-8"?>
-<layoutRules xmlns="https://swooshz.com/kqag/layout-rules/v1" schema="swooshz.quote-layout-rules.v1">
+<file path=customXml/sqag-layout-rules.xml><?xml version="1.0" encoding="utf-8"?>
+<layoutRules xmlns="https://swooshz.com/sqag/layout-rules/v1" schema="swooshz.quote-layout-rules.v1">
   <json>{"company_details":{"align_details_to_logo_left":true,"blank_line_before_bank_detail":true,"details_alignment":"left","details_below_logo":true,"details_first_page_only":true,"details_font_size_pt":9,"keep_logo_and_details_inside_print_area":true,"print_area_columns":"A:I"},"header":{"client_block":{"alignment":"left","fields":["client.name","client.address","client.attention","client.title","quote_date","project.title"],"position":"top-left"},"company_block":{"alignment":"left","position":"top-right","repeat_logo_on_continuation_pages":true,"show_details_on_first_page_only":true}},"line_items":{"bold_headers":true,"columns":["Pos.","Quantity","Service","Estimate"],"detail_rows":{"allowed_display_prices":["numeric","FOC","Included"],"number_format":"0.0"},"estimate_alignment":"right","numeric_price_format":"#,##0.00","quantity_alignment":"center","quantity_column_must_fit_examples":["24 m length","36 sqm"],"section_rows":{"amount_mode":"itemized_by_default","number_format":"0.0"},"show_internal_costs":false,"square_metre_unit":"sqm"},"output":{"currency":"SGD","master_format":"xlsx","pdf_default":"disabled"},"profile_id":"default","schema_version":1,"security":{"escape_formula_prefixes":["'=","'+","'-","'@"],"frontend_exposes_internal_pricing":false,"treat_text_as_untrusted_spreadsheet_text":true},"template":{"print_area_columns":"A:I","workbook":"quotation-layout.xlsx","worksheet":"Quotation"},"terms_notes_signature":{"acceptance_block_separate_from_notes":true,"company_signatory_title_below_name":true,"customer_acceptance_text_separate_from_terms":true,"notes_numbering":"plain_sequential","payment_terms_bold":true,"signature_blocks":["company","customer"]},"totals":{"border_scope":["label","amount","currency"],"keep_rows_together":true,"labels":["Total","Quote-level tax label and rate","Total including selected tax label"],"use_strong_bottom_rule_under_final_total":true,"use_top_rule_above_final_total":true,"use_top_rule_above_total":true}}</json>
 </layoutRules>
 </file>
</xml_diff>